<commit_message>
Update HotelAI data to v8 (final): merged tickets, calls demo data, verification codes, discounts, hotel photos, Maintenance
</commit_message>
<xml_diff>
--- a/evaluation/egyptian_review.xlsx
+++ b/evaluation/egyptian_review.xlsx
@@ -557,11 +557,11 @@
     <row r="11" ht="15" customHeight="1" s="7">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>FAQ_Answers (215)</t>
+          <t>FAQ_Answers (218)</t>
         </is>
       </c>
       <c r="B11" s="9">
-        <f>COUNTIF(FAQ_Answers!H2:H216,"تمام")&amp;" / "&amp;COUNTIF(FAQ_Answers!H2:H216,"محتاج تعديل")&amp;" / "&amp;COUNTIF(FAQ_Answers!H2:H216,"مش متأكد")&amp;" / "&amp;COUNTBLANK(FAQ_Answers!H2:H216)</f>
+        <f>COUNTIF(FAQ_Answers!H2:H219,"تمام")&amp;" / "&amp;COUNTIF(FAQ_Answers!H2:H219,"محتاج تعديل")&amp;" / "&amp;COUNTIF(FAQ_Answers!H2:H219,"مش متأكد")&amp;" / "&amp;COUNTBLANK(FAQ_Answers!H2:H219)</f>
         <v/>
       </c>
     </row>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K216"/>
+  <dimension ref="A1:K219"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="6" min="1" max="1"/>
@@ -9227,10 +9227,127 @@
       <c r="J216" s="12" t="n"/>
       <c r="K216" s="12" t="n"/>
     </row>
+    <row r="217">
+      <c r="A217" s="9" t="inlineStr">
+        <is>
+          <t>E216</t>
+        </is>
+      </c>
+      <c r="B217" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C217" s="9" t="inlineStr">
+        <is>
+          <t>INT034</t>
+        </is>
+      </c>
+      <c r="D217" s="9" t="inlineStr">
+        <is>
+          <t>FAQ3986</t>
+        </is>
+      </c>
+      <c r="E217" s="9" t="inlineStr">
+        <is>
+          <t>إزاي أعمل حساب على الموقع بتاعكم؟</t>
+        </is>
+      </c>
+      <c r="F217" s="9" t="inlineStr">
+        <is>
+          <t>سجّل في موقع الفندق بإيميلك وباسورد، وهيوصلك كود من 6 أرقام تأكّد بيه الإيميل: شغال مرة واحدة لمدة 10 دقايق، وليك 5 محاولات بالكتير. وبعد ما تعمل لوجين تقدر تحجز وتتابع حجوزاتك.</t>
+        </is>
+      </c>
+      <c r="G217" s="9" t="inlineStr">
+        <is>
+          <t>سجّل في موقع الفندق ببريدك الإلكتروني وكلمة مرور، وسنرسل إليك رمزاً من 6 أرقام لتأكيد البريد: يُستخدم مرة واحدة خلال 10 دقائق، مع 5 محاولات كحد أقصى. وبعد تسجيل الدخول يمكنك الحجز وإدارة حجوزاتك.</t>
+        </is>
+      </c>
+      <c r="H217" s="12" t="n"/>
+      <c r="I217" s="12" t="n"/>
+      <c r="J217" s="12" t="n"/>
+      <c r="K217" s="12" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="9" t="inlineStr">
+        <is>
+          <t>E217</t>
+        </is>
+      </c>
+      <c r="B218" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C218" s="9" t="inlineStr">
+        <is>
+          <t>INT034</t>
+        </is>
+      </c>
+      <c r="D218" s="9" t="inlineStr">
+        <is>
+          <t>FAQ3991</t>
+        </is>
+      </c>
+      <c r="E218" s="9" t="inlineStr">
+        <is>
+          <t>نسيت الباسورد بتاعي، أعمل إيه؟</t>
+        </is>
+      </c>
+      <c r="F218" s="9" t="inlineStr">
+        <is>
+          <t>دوس على «نسيت الباسورد» في صفحة الدخول، وهيوصلك كود من 6 أرقام على إيميل الحساب: شغال مرة واحدة لمدة 10 دقايق، وليك 5 محاولات بالكتير، وبعدها تعمل باسورد جديد. والفندق عمره ما بيطلب منك الباسورد في تليفون أو شات أو إيميل.</t>
+        </is>
+      </c>
+      <c r="G218" s="9" t="inlineStr">
+        <is>
+          <t>اختر «نسيت كلمة المرور» في صفحة الدخول، فيصلك رمز من 6 أرقام على بريد حسابك: يُستخدم مرة واحدة خلال 10 دقائق، مع 5 محاولات كحد أقصى، ثم تضع كلمة مرور جديدة. ولا يطلب الفندق كلمة المرور أبداً بالهاتف أو المحادثة أو البريد الإلكتروني.</t>
+        </is>
+      </c>
+      <c r="H218" s="12" t="n"/>
+      <c r="I218" s="12" t="n"/>
+      <c r="J218" s="12" t="n"/>
+      <c r="K218" s="12" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="9" t="inlineStr">
+        <is>
+          <t>E218</t>
+        </is>
+      </c>
+      <c r="B219" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C219" s="9" t="inlineStr">
+        <is>
+          <t>INT034</t>
+        </is>
+      </c>
+      <c r="D219" s="9" t="inlineStr">
+        <is>
+          <t>FAQ3996</t>
+        </is>
+      </c>
+      <c r="E219" s="9" t="inlineStr">
+        <is>
+          <t>لازم أعمل حساب عشان أحجز مع المساعد بتاعكم؟</t>
+        </is>
+      </c>
+      <c r="F219" s="9" t="inlineStr">
+        <is>
+          <t>أيوه. من غير لوجين تقدر تسأل أي سؤال عام عن الفندق، لكن الحجز أو إنك تشوف حجز أو تعدّله أو تطلب حاجة محتاج لوجين الأول، وبعدها تقدر تضيف حجز عملته بالتليفون أو من شركة سياحة أو موقع حجز برقمه واسم العيلة اللي عليه. ولو في طوارئ المساعد بيساعدك على طول، عامل لوجين أو لأ.</t>
+        </is>
+      </c>
+      <c r="G219" s="9" t="inlineStr">
+        <is>
+          <t>نعم. دون تسجيل الدخول يمكنك طرح الأسئلة العامة عن الفندق، أما الحجز أو الاطلاع على حجز أو تعديله أو تقديم طلب فيحتاج إلى تسجيل الدخول أولاً، ويمكن بعدها إضافة حجز تم بالهاتف أو عبر وكالة أو منصة حجز برقمه واسم العائلة المسجل عليه. وفي حالات الطوارئ يساعدك المساعد فوراً، سجّلت الدخول أم لا.</t>
+        </is>
+      </c>
+      <c r="H219" s="12" t="n"/>
+      <c r="I219" s="12" t="n"/>
+      <c r="J219" s="12" t="n"/>
+      <c r="K219" s="12" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K216"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H216" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="H2:H219" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"تمام,محتاج تعديل,مش متأكد"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -14434,7 +14551,7 @@
       </c>
       <c r="B185" s="9" t="inlineStr">
         <is>
-          <t>INT012_F3</t>
+          <t>INT012_F6_visitor_login</t>
         </is>
       </c>
       <c r="C185" s="9" t="n">
@@ -14442,12 +14559,12 @@
       </c>
       <c r="D185" s="9" t="inlineStr">
         <is>
-          <t>في مستويات مختلفة في البرنامج؟</t>
+          <t>أنا معايا كام نقطة في برنامج الولاء؟</t>
         </is>
       </c>
       <c r="E185" s="9" t="inlineStr">
         <is>
-          <t>في 4 مستويات: العادي أول ما تشترك، والفضي بعد 10 ليالي، والدهبي بعد 25، والبلاتيني بعد 50 ليلة في السنة.</t>
+          <t>علشان أشوف نقطك لازم تسجّل دخول الأول من موقع الفندق. ولو مش عامل حساب تقدر تعمله بإيميلك، وهيوصلك كود من 6 أرقام تأكّده بيه.</t>
         </is>
       </c>
       <c r="F185" s="12" t="n"/>
@@ -14462,7 +14579,7 @@
       </c>
       <c r="B186" s="9" t="inlineStr">
         <is>
-          <t>INT012_F3</t>
+          <t>INT012_F6_visitor_login</t>
         </is>
       </c>
       <c r="C186" s="9" t="n">
@@ -14470,12 +14587,12 @@
       </c>
       <c r="D186" s="9" t="inlineStr">
         <is>
-          <t>والأعضاء بياخدوا إيه؟</t>
+          <t>ولو نسيت الباسورد؟</t>
         </is>
       </c>
       <c r="E186" s="9" t="inlineStr">
         <is>
-          <t>الفضي: خروج لحد 1 الضهر. الدهبي: لحد 2 الضهر وترقية للأوضة وخصم 10% في السبا. البلاتيني: لحد 4 العصر وفطار ببلاش لاتنين وأولوية في الترقية وخصم 15% في السبا، وكله على حسب المتاح.</t>
+          <t>دوس على «نسيت الباسورد» في صفحة الدخول، وهيوصلك كود على الإيميل شغال 10 دقايق، وبعدها تعمل باسورد جديد.</t>
         </is>
       </c>
       <c r="F186" s="12" t="n"/>
@@ -14490,7 +14607,7 @@
       </c>
       <c r="B187" s="9" t="inlineStr">
         <is>
-          <t>INT012_F3</t>
+          <t>INT012_F6_visitor_login</t>
         </is>
       </c>
       <c r="C187" s="9" t="n">
@@ -14518,7 +14635,7 @@
       </c>
       <c r="B188" s="9" t="inlineStr">
         <is>
-          <t>INT012_F3</t>
+          <t>INT027_F2_discount_request</t>
         </is>
       </c>
       <c r="C188" s="9" t="n">
@@ -14526,12 +14643,12 @@
       </c>
       <c r="D188" s="9" t="inlineStr">
         <is>
-          <t>العضوية مقسمة إزاي؟</t>
+          <t>ممكن تعملولي خصم على الإقامة الجاية؟</t>
         </is>
       </c>
       <c r="E188" s="9" t="inlineStr">
         <is>
-          <t>في 4 مستويات: العادي أول ما تشترك، والفضي بعد 10 ليالي، والدهبي بعد 25، والبلاتيني بعد 50 ليلة في السنة.</t>
+          <t>على السعر المرن أقدر أطبّق خصم الإقامة الطويلة 12% لو 7 ليالي أو أكتر، أو كود خصم ساري. غير كده الفندق هو اللي بيقرر: أقدر أبعت طلب خصم، ولو اتوافق عليه هيوصلك كود شخصي على الإيميل. أبعته؟</t>
         </is>
       </c>
       <c r="F188" s="12" t="n"/>
@@ -14546,7 +14663,7 @@
       </c>
       <c r="B189" s="9" t="inlineStr">
         <is>
-          <t>INT012_F3</t>
+          <t>INT027_F2_discount_request</t>
         </is>
       </c>
       <c r="C189" s="9" t="n">
@@ -14554,12 +14671,12 @@
       </c>
       <c r="D189" s="9" t="inlineStr">
         <is>
-          <t>والأعضاء بياخدوا إيه؟</t>
+          <t>آه ياريت، هي 4 ليالي في يناير.</t>
         </is>
       </c>
       <c r="E189" s="9" t="inlineStr">
         <is>
-          <t>الفضي: خروج لحد 1 الضهر. الدهبي: لحد 2 الضهر وترقية للأوضة وخصم 10% في السبا. البلاتيني: لحد 4 العصر وفطار ببلاش لاتنين وأولوية في الترقية وخصم 15% في السبا، وكله على حسب المتاح.</t>
+          <t>تمام، بعت طلب الخصم لـ 4 ليالي في يناير، والرد هيوصلك على الإيميل.</t>
         </is>
       </c>
       <c r="F189" s="12" t="n"/>
@@ -14574,7 +14691,7 @@
       </c>
       <c r="B190" s="9" t="inlineStr">
         <is>
-          <t>INT012_F3</t>
+          <t>INT027_F2_discount_request</t>
         </is>
       </c>
       <c r="C190" s="9" t="n">
@@ -16379,7 +16496,7 @@
       </c>
       <c r="E254" s="9" t="inlineStr">
         <is>
-          <t>كلّم الاستقبال من تليفون الأوضة حالاً، الفندق يقدر يجيب دكتور أو إسعاف. ولو الحالة خطر على الحياة كلّم الطوارئ على طول. انت في أوضة كام؟</t>
+          <t>لو الحالة خطر على الحياة كلّم الإسعاف على 123 حالاً. أنا بلّغت فريق الفندق إن في حالة طوارئ، ورقم الاستقبال ‎+20 2 2794 5500. حضرتك في أوضة كام؟</t>
         </is>
       </c>
       <c r="F254" s="12" t="n"/>
@@ -16407,7 +16524,7 @@
       </c>
       <c r="E255" s="9" t="inlineStr">
         <is>
-          <t>الاستقبال اتبلغ بأوضة 1506 والمساعدة جاية في الطريق. وفي إسعافات أولية في الاستقبال.</t>
+          <t>تمام، في حد من الموظفين طالع لأوضة 1506 دلوقتي، والفندق يقدر يجيب دكتور. خليك جنبه وسيب الباب من غير قفل.</t>
         </is>
       </c>
       <c r="F255" s="12" t="n"/>
@@ -16435,7 +16552,7 @@
       </c>
       <c r="E256" s="9" t="inlineStr">
         <is>
-          <t>كلّم الاستقبال من تليفون الأوضة حالاً، الفندق يقدر يجيب دكتور أو إسعاف. ولو الحالة خطر على الحياة كلّم الطوارئ على طول. انت في أوضة كام؟</t>
+          <t>لو الحالة خطر على الحياة كلّم الإسعاف على 123 حالاً. أنا بلّغت فريق الفندق إن في حالة طوارئ، ورقم الاستقبال ‎+20 2 2794 5500. حضرتك في أوضة كام؟</t>
         </is>
       </c>
       <c r="F256" s="12" t="n"/>
@@ -16463,7 +16580,7 @@
       </c>
       <c r="E257" s="9" t="inlineStr">
         <is>
-          <t>الاستقبال اتبلغ بأوضة 807 والمساعدة جاية في الطريق. وفي إسعافات أولية في الاستقبال.</t>
+          <t>تمام، في حد من الموظفين طالع لأوضة 807 دلوقتي، والفندق يقدر يجيب دكتور. خليك جنبه وسيب الباب من غير قفل.</t>
         </is>
       </c>
       <c r="F257" s="12" t="n"/>
@@ -16491,7 +16608,7 @@
       </c>
       <c r="E258" s="9" t="inlineStr">
         <is>
-          <t>كلّم الاستقبال من تليفون الأوضة حالاً، الفندق يقدر يجيب دكتور أو إسعاف. ولو الحالة خطر على الحياة كلّم الطوارئ على طول. انت في أوضة كام؟</t>
+          <t>لو الحالة خطر على الحياة كلّم الإسعاف على 123 حالاً. أنا بلّغت فريق الفندق إن في حالة طوارئ، ورقم الاستقبال ‎+20 2 2794 5500. حضرتك في أوضة كام؟</t>
         </is>
       </c>
       <c r="F258" s="12" t="n"/>
@@ -16519,7 +16636,7 @@
       </c>
       <c r="E259" s="9" t="inlineStr">
         <is>
-          <t>الاستقبال اتبلغ بأوضة 1402 والمساعدة جاية في الطريق. وفي إسعافات أولية في الاستقبال.</t>
+          <t>تمام، في حد من الموظفين طالع لأوضة 1402 دلوقتي، والفندق يقدر يجيب دكتور. خليك جنبه وسيب الباب من غير قفل.</t>
         </is>
       </c>
       <c r="F259" s="12" t="n"/>
@@ -16743,7 +16860,7 @@
       </c>
       <c r="E267" s="9" t="inlineStr">
         <is>
-          <t>الاستقبال والأمن اتبلغوا بأوضة 1507 وجايين لك. لحد ما ييجوا اقفل الباب واستخدم الخزنة للحاجات الغالية.</t>
+          <t>الاستقبال والأمن اتبلغوا بأوضة 1507 وجايين لك. لحد ما ييجوا اقفل الباب واستخدم الخزنة للحاجات الغالية. وتقدر كمان تبلّغ البوليس على 122.</t>
         </is>
       </c>
       <c r="F267" s="12" t="n"/>
@@ -16799,7 +16916,7 @@
       </c>
       <c r="E269" s="9" t="inlineStr">
         <is>
-          <t>الاستقبال والأمن اتبلغوا بأوضة 1407 وجايين لك. لحد ما ييجوا اقفل الباب واستخدم الخزنة للحاجات الغالية.</t>
+          <t>الاستقبال والأمن اتبلغوا بأوضة 1407 وجايين لك. لحد ما ييجوا اقفل الباب واستخدم الخزنة للحاجات الغالية. وتقدر كمان تبلّغ البوليس على 122.</t>
         </is>
       </c>
       <c r="F269" s="12" t="n"/>
@@ -16855,7 +16972,7 @@
       </c>
       <c r="E271" s="9" t="inlineStr">
         <is>
-          <t>الاستقبال والأمن اتبلغوا بأوضة 1405 وجايين لك. لحد ما ييجوا اقفل الباب واستخدم الخزنة للحاجات الغالية.</t>
+          <t>الاستقبال والأمن اتبلغوا بأوضة 1405 وجايين لك. لحد ما ييجوا اقفل الباب واستخدم الخزنة للحاجات الغالية. وتقدر كمان تبلّغ البوليس على 122.</t>
         </is>
       </c>
       <c r="F271" s="12" t="n"/>
@@ -17051,7 +17168,7 @@
       </c>
       <c r="E278" s="9" t="inlineStr">
         <is>
-          <t>اخرج دلوقتي من مخارج الطوارئ اللي عليها علامات واتبع تعليمات الموظفين. انزل على السلم مش الأسانسير، وروح نقطة التجمع.</t>
+          <t>اخرج دلوقتي من مخارج الطوارئ اللي عليها علامات، وانزل على السلم مش الأسانسير، وروح نقطة التجمع. أنا بلّغت فريق الفندق، ولو شفت نار كلّم المطافي على 180. الاستقبال: ‎+20 2 2794 5500.</t>
         </is>
       </c>
       <c r="F278" s="12" t="n"/>
@@ -17107,7 +17224,7 @@
       </c>
       <c r="E280" s="9" t="inlineStr">
         <is>
-          <t>اخرج دلوقتي من مخارج الطوارئ اللي عليها علامات واتبع تعليمات الموظفين. انزل على السلم مش الأسانسير، وروح نقطة التجمع.</t>
+          <t>اخرج دلوقتي من مخارج الطوارئ اللي عليها علامات، وانزل على السلم مش الأسانسير، وروح نقطة التجمع. أنا بلّغت فريق الفندق، ولو شفت نار كلّم المطافي على 180. الاستقبال: ‎+20 2 2794 5500.</t>
         </is>
       </c>
       <c r="F280" s="12" t="n"/>
@@ -17163,7 +17280,7 @@
       </c>
       <c r="E282" s="9" t="inlineStr">
         <is>
-          <t>اخرج دلوقتي من مخارج الطوارئ اللي عليها علامات واتبع تعليمات الموظفين. انزل على السلم مش الأسانسير، وروح نقطة التجمع.</t>
+          <t>اخرج دلوقتي من مخارج الطوارئ اللي عليها علامات، وانزل على السلم مش الأسانسير، وروح نقطة التجمع. أنا بلّغت فريق الفندق، ولو شفت نار كلّم المطافي على 180. الاستقبال: ‎+20 2 2794 5500.</t>
         </is>
       </c>
       <c r="F282" s="12" t="n"/>
@@ -19263,7 +19380,7 @@
       </c>
       <c r="E357" s="9" t="inlineStr">
         <is>
-          <t>آسف، ماقدرتش أفهمك صح. وبدل ما أخمن للمرة التالتة هحوّلك لحد من فريق الفندق.</t>
+          <t>أنا آسفة، ماقدرتش أفهم حضرتك صح. وبدل ما أخمّن للمرة التالتة، تحب أوصّلك بحد من فريق الفندق هنا في الشات؟</t>
         </is>
       </c>
       <c r="F357" s="12" t="n"/>
@@ -19286,12 +19403,12 @@
       </c>
       <c r="D358" s="9" t="inlineStr">
         <is>
-          <t>أخيراً. هياخد قد إيه؟</t>
+          <t>أيوه ياريت. هياخد قد إيه؟</t>
         </is>
       </c>
       <c r="E358" s="9" t="inlineStr">
         <is>
-          <t>الاستقبال موجود 24 ساعة، فيه حد متاح دلوقتي. ولو مش عايز تستنى هنا تقدر تكلم الاستقبال على طول وهيكون معاهم تفاصيل المحادثة دي.</t>
+          <t>في حد من الموظفين بيدخل الشات دلوقتي وهيشوف كلامنا من الأول، فمش هتحتاج تعيد حاجة.</t>
         </is>
       </c>
       <c r="F358" s="12" t="n"/>

</xml_diff>